<commit_message>
chore: sync Stata-Tools releases and regenerated demos
Publish gcomp 2.0.0 and iivw 4.0.0, syncing their .ado, .pkg,
.sthlp, and README metadata. Regenerate datamap 1.6.7 demo datasets
and outputs, including decimal formatting and privacy console capture.
Simplify diagtab's check_xlsx.py and refresh demo_diagtab.xlsx. Correct
the package catalog to list tabtools 2.0.0 instead of 2.1.0.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_table1.xlsx
+++ b/tabtools/demo/demo_table1.xlsx
@@ -14,9 +14,9 @@
     <sheet name="Table 1 Formats" sheetId="6" r:id="rId8"/>
     <sheet name="Table 1 Missing" sheetId="7" r:id="rId9"/>
     <sheet name="Table 1 Custom" sheetId="8" r:id="rId10"/>
-    <sheet name="Table 1 NEJM" sheetId="9" r:id="rId11"/>
-    <sheet name="Theme BMJ" sheetId="10" r:id="rId12"/>
-    <sheet name="Theme APA" sheetId="11" r:id="rId13"/>
+    <sheet name="Table 1 Compact" sheetId="9" r:id="rId11"/>
+    <sheet name="Explicit Arial" sheetId="10" r:id="rId12"/>
+    <sheet name="Explicit Serif" sheetId="11" r:id="rId13"/>
     <sheet name="Small Cells Primary" sheetId="12" r:id="rId14"/>
     <sheet name="Small Cells Complement" sheetId="13" r:id="rId15"/>
     <sheet name="Small Cells Binary" sheetId="14" r:id="rId16"/>
@@ -763,13 +763,13 @@
     <t>SD shown as mean [SD]. IQR uses 'to' separator. Row % for categoricals.</t>
   </si>
   <si>
-    <t>Table 1. Baseline Characteristics (NEJM Style)</t>
-  </si>
-  <si>
-    <t>Table 1. Baseline Characteristics (BMJ Style)</t>
-  </si>
-  <si>
-    <t>Table 1. Baseline Characteristics (APA Style)</t>
+    <t>Table 1. Baseline Characteristics (Compact Style)</t>
+  </si>
+  <si>
+    <t>Table 1. Baseline Characteristics (Arial Style)</t>
+  </si>
+  <si>
+    <t>Table 1. Baseline Characteristics (Serif Style)</t>
   </si>
   <si>
     <t>Small-cell suppression: primary counts only</t>

</xml_diff>

<commit_message>
fix(tabtools): resolve correctness issues and bump to 2.1.10
Address parsing and output correctness edge cases across estimation,
table aggregation, and export routines. regtab.ado parses model scale
strictly from options after top-level commas to avoid misinterpreting
covariates or abbreviations; hrcomptab.ado matches estimates by label
instead of position; desctab.ado and _desctab_collect.ado preserve
quoted labels, bound categorical SMDs to pairwise levels, and drop
the r(table) row limit; puttab.ado evaluates if/in inside frame()
sources and exports %t dates as dates. Bump tabtools to version
2.1.10 and sync all .ado, .sthlp, and README.md files.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_table1.xlsx
+++ b/tabtools/demo/demo_table1.xlsx
@@ -394,7 +394,7 @@
     <t>Table 1. Baseline Characteristics with Balance Diagnostics</t>
   </si>
   <si>
-    <t>No. (Column %), and Mean±SD or Geometric mean (×/GSD), and Median (Q1, Q3)</t>
+    <t>No. (Column %), Mean±SD, Geometric mean (×/GSD), or Median (Q1, Q3)</t>
   </si>
   <si>
     <t>C-reactive protein (mg/L)</t>
@@ -505,7 +505,7 @@
     <t>Table 1. Alternative Formatting Options Demo</t>
   </si>
   <si>
-    <t>Column % (No.), and Mean±SD or Geometric mean (×/GSD), and Median (Q1, Q3)</t>
+    <t>Column % (No.), Mean±SD, Geometric mean (×/GSD), or Median (Q1, Q3)</t>
   </si>
   <si>
     <t>Age at cohort entry (years), mean±SD</t>
@@ -682,7 +682,7 @@
     <t>Table 1. Custom Symbol Formatting Demo</t>
   </si>
   <si>
-    <t>No. (Row %) or No. (Column %), and Mean [SD] or Geometric mean (×/GSD), and Median (Q1 to Q3)</t>
+    <t>No. (Row %), No. (Column %), Mean [SD], Geometric mean (×/GSD), or Median (Q1 to Q3)</t>
   </si>
   <si>
     <t>58.3 [13.4]</t>
@@ -4056,7 +4056,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
-    <col min="2" max="2" width="43.11328125" style="1" customWidth="true"/>
+    <col min="2" max="2" width="40.7109375" style="1" customWidth="true"/>
     <col min="3" max="3" width="12.7109375" style="1" customWidth="true"/>
     <col min="4" max="4" width="12.7109375" style="1" customWidth="true"/>
     <col min="7" max="7" width="10.7109375" style="1" customWidth="true"/>
@@ -5071,7 +5071,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
-    <col min="2" max="2" width="42.51171875" style="1" customWidth="true"/>
+    <col min="2" max="2" width="40.11328125" style="1" customWidth="true"/>
     <col min="3" max="3" width="12.7109375" style="1" customWidth="true"/>
     <col min="4" max="4" width="12.7109375" style="1" customWidth="true"/>
     <col min="5" max="5" width="10.7109375" style="1" customWidth="true"/>
@@ -5390,7 +5390,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
-    <col min="2" max="2" width="48.51171875" style="1" customWidth="true"/>
+    <col min="2" max="2" width="45.7109375" style="1" customWidth="true"/>
     <col min="3" max="3" width="16.7109375" style="1" customWidth="true"/>
     <col min="4" max="4" width="16.7109375" style="1" customWidth="true"/>
     <col min="5" max="5" width="10.7109375" style="1" customWidth="true"/>

</xml_diff>